<commit_message>
TGZ2resolver page in progress
</commit_message>
<xml_diff>
--- a/docs/Manual/source/tab/parameters.en.xlsx
+++ b/docs/Manual/source/tab/parameters.en.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="35"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="44"/>
   </bookViews>
   <sheets>
     <sheet name="TGZ-D-48-13_26" sheetId="1" state="visible" r:id="rId3"/>
@@ -52,7 +52,8 @@
     <sheet name="X8_commonHW_DI_RI_tab" sheetId="42" state="visible" r:id="rId44"/>
     <sheet name="X8_commonHW_DO_tab" sheetId="43" state="visible" r:id="rId45"/>
     <sheet name="X8_commonHW_AI_tab" sheetId="44" state="visible" r:id="rId46"/>
-    <sheet name="TGmonitor7" sheetId="45" state="visible" r:id="rId47"/>
+    <sheet name="X16_commonHW_RES_tab" sheetId="45" state="visible" r:id="rId47"/>
+    <sheet name="TGmonitor7" sheetId="46" state="visible" r:id="rId48"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2251" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2269" uniqueCount="362">
   <si>
     <t xml:space="preserve">POWER SUPPLY</t>
   </si>
@@ -1070,6 +1071,51 @@
     <t xml:space="preserve">us</t>
   </si>
   <si>
+    <t xml:space="preserve">Parameter No.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feedback type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-ResolverPoles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2~42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of resolver poles (2 = 1 polepair)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-Observer_K1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">‰</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtrační constant 1 – set to 50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-Observer_K2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtrační constant 2 – set to 1000</t>
+  </si>
+  <si>
     <t xml:space="preserve">Supply voltage </t>
   </si>
   <si>
@@ -1142,7 +1188,7 @@
     <numFmt numFmtId="165" formatCode="0.00\ %"/>
     <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1171,6 +1217,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1216,7 +1268,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1235,6 +1287,14 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -10686,6 +10746,117 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="39"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>340</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -10704,7 +10875,7 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>248</v>
@@ -10712,10 +10883,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -10745,7 +10916,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>265</v>
@@ -10754,7 +10925,7 @@
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>1</v>
@@ -10762,66 +10933,66 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>332</v>
+        <v>347</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>334</v>
+        <v>349</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>342</v>
+        <v>356</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>346</v>
+        <v>360</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>361</v>
       </c>
     </row>
   </sheetData>

</xml_diff>